<commit_message>
hmm looking at outliers this time how fun! distribution of counts and dex vs tcr beta with spearman specificity_correlations also hypothesising about different ways of looking at levenshtein
</commit_message>
<xml_diff>
--- a/Final_Figures_and_Sheets_Singleset/Kb_jgene_decomposition_CDR3a.xlsx
+++ b/Final_Figures_and_Sheets_Singleset/Kb_jgene_decomposition_CDR3a.xlsx
@@ -1560,10 +1560,10 @@
         <v>0.005227781926811053</v>
       </c>
       <c r="C32" t="n">
-        <v>0.005227781926811053</v>
+        <v>0.005227781926811052</v>
       </c>
       <c r="D32" t="n">
-        <v>0</v>
+        <v>8.673617379884035e-19</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1923,7 +1923,7 @@
         <v>0.02267290126141801</v>
       </c>
       <c r="D42" t="n">
-        <v>-3.469446951953614e-18</v>
+        <v>0</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -2028,10 +2028,10 @@
         <v>0.00931430836305985</v>
       </c>
       <c r="C45" t="n">
-        <v>0.00931430836305985</v>
+        <v>0.009314308363059848</v>
       </c>
       <c r="D45" t="n">
-        <v>0</v>
+        <v>1.734723475976807e-18</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -2067,7 +2067,7 @@
         <v>0.01087958694449567</v>
       </c>
       <c r="D46" t="n">
-        <v>0</v>
+        <v>-3.469446951953614e-18</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -2964,10 +2964,10 @@
         <v>0.006896551724137931</v>
       </c>
       <c r="C71" t="n">
-        <v>0.00689655172413793</v>
+        <v>0.006896551724137929</v>
       </c>
       <c r="D71" t="n">
-        <v>8.673617379884035e-19</v>
+        <v>1.734723475976807e-18</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -3039,7 +3039,7 @@
         <v>0.01865847897968824</v>
       </c>
       <c r="D73" t="n">
-        <v>3.469446951953614e-18</v>
+        <v>0</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -3075,7 +3075,7 @@
         <v>0.002130681818181818</v>
       </c>
       <c r="D74" t="n">
-        <v>0</v>
+        <v>-4.336808689942018e-19</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -3288,10 +3288,10 @@
         <v>0.009529411764705882</v>
       </c>
       <c r="C80" t="n">
-        <v>0.009529411764705882</v>
+        <v>0.009529411764705883</v>
       </c>
       <c r="D80" t="n">
-        <v>0</v>
+        <v>-1.734723475976807e-18</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -3492,10 +3492,10 @@
         <v>0.005227781926811053</v>
       </c>
       <c r="C86" t="n">
-        <v>0.005227781926811053</v>
+        <v>0.005227781926811052</v>
       </c>
       <c r="D86" t="n">
-        <v>0</v>
+        <v>8.673617379884035e-19</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -4103,7 +4103,7 @@
         <v>0.02267290126141801</v>
       </c>
       <c r="D105" t="n">
-        <v>-3.469446951953614e-18</v>
+        <v>0</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -4484,10 +4484,10 @@
         <v>0.00931430836305985</v>
       </c>
       <c r="C117" t="n">
-        <v>0.00931430836305985</v>
+        <v>0.009314308363059848</v>
       </c>
       <c r="D117" t="n">
-        <v>0</v>
+        <v>1.734723475976807e-18</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -4519,7 +4519,7 @@
         <v>0.01087958694449567</v>
       </c>
       <c r="D118" t="n">
-        <v>0</v>
+        <v>-3.469446951953614e-18</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -4775,7 +4775,7 @@
         <v>0.003572615486872715</v>
       </c>
       <c r="D126" t="n">
-        <v>0</v>
+        <v>4.336808689942018e-19</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -5988,10 +5988,10 @@
         <v>0.006896551724137931</v>
       </c>
       <c r="C164" t="n">
-        <v>0.00689655172413793</v>
+        <v>0.006896551724137929</v>
       </c>
       <c r="D164" t="n">
-        <v>8.673617379884035e-19</v>
+        <v>1.734723475976807e-18</v>
       </c>
       <c r="E164" t="inlineStr">
         <is>
@@ -6055,7 +6055,7 @@
         <v>0.01865847897968824</v>
       </c>
       <c r="D166" t="n">
-        <v>3.469446951953614e-18</v>
+        <v>0</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
@@ -6183,7 +6183,7 @@
         <v>0.002130681818181818</v>
       </c>
       <c r="D170" t="n">
-        <v>0</v>
+        <v>-4.336808689942018e-19</v>
       </c>
       <c r="E170" t="inlineStr">
         <is>
@@ -6756,10 +6756,10 @@
         <v>0.009529411764705882</v>
       </c>
       <c r="C188" t="n">
-        <v>0.009529411764705882</v>
+        <v>0.009529411764705883</v>
       </c>
       <c r="D188" t="n">
-        <v>0</v>
+        <v>-1.734723475976807e-18</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -6948,10 +6948,10 @@
         <v>0.005227781926811053</v>
       </c>
       <c r="C194" t="n">
-        <v>0.005227781926811053</v>
+        <v>0.005227781926811052</v>
       </c>
       <c r="D194" t="n">
-        <v>0</v>
+        <v>8.673617379884035e-19</v>
       </c>
       <c r="E194" t="inlineStr"/>
       <c r="F194" t="inlineStr">
@@ -7140,10 +7140,10 @@
         <v>0.02894642215030565</v>
       </c>
       <c r="C200" t="n">
-        <v>0.02894642215030565</v>
+        <v>0.02894642215030564</v>
       </c>
       <c r="D200" t="n">
-        <v>0</v>
+        <v>3.469446951953614e-18</v>
       </c>
       <c r="E200" t="inlineStr"/>
       <c r="F200" t="inlineStr">
@@ -8164,10 +8164,10 @@
         <v>0.0004001600640256103</v>
       </c>
       <c r="C232" t="n">
-        <v>0.0004001600640256103</v>
+        <v>0.0004001600640256102</v>
       </c>
       <c r="D232" t="n">
-        <v>0</v>
+        <v>5.421010862427522e-20</v>
       </c>
       <c r="E232" t="inlineStr"/>
       <c r="F232" t="inlineStr">
@@ -8423,7 +8423,7 @@
         <v>0.02267290126141801</v>
       </c>
       <c r="D240" t="n">
-        <v>-3.469446951953614e-18</v>
+        <v>0</v>
       </c>
       <c r="E240" t="inlineStr"/>
       <c r="F240" t="inlineStr">
@@ -8519,7 +8519,7 @@
         <v>0.001479289940828402</v>
       </c>
       <c r="D243" t="n">
-        <v>0</v>
+        <v>2.168404344971009e-19</v>
       </c>
       <c r="E243" t="inlineStr"/>
       <c r="F243" t="inlineStr">
@@ -11460,10 +11460,10 @@
         <v>0.006896551724137931</v>
       </c>
       <c r="C335" t="n">
-        <v>0.00689655172413793</v>
+        <v>0.006896551724137929</v>
       </c>
       <c r="D335" t="n">
-        <v>8.673617379884035e-19</v>
+        <v>1.734723475976807e-18</v>
       </c>
       <c r="E335" t="inlineStr"/>
       <c r="F335" t="inlineStr">
@@ -11527,7 +11527,7 @@
         <v>0.01865847897968824</v>
       </c>
       <c r="D337" t="n">
-        <v>3.469446951953614e-18</v>
+        <v>0</v>
       </c>
       <c r="E337" t="inlineStr"/>
       <c r="F337" t="inlineStr">
@@ -11559,7 +11559,7 @@
         <v>0.002130681818181818</v>
       </c>
       <c r="D338" t="n">
-        <v>0</v>
+        <v>-4.336808689942018e-19</v>
       </c>
       <c r="E338" t="inlineStr"/>
       <c r="F338" t="inlineStr">
@@ -11780,10 +11780,10 @@
         <v>0.00931430836305985</v>
       </c>
       <c r="C345" t="n">
-        <v>0.00931430836305985</v>
+        <v>0.009314308363059848</v>
       </c>
       <c r="D345" t="n">
-        <v>0</v>
+        <v>1.734723475976807e-18</v>
       </c>
       <c r="E345" t="inlineStr"/>
       <c r="F345" t="inlineStr">
@@ -12007,7 +12007,7 @@
         <v>0.01087958694449567</v>
       </c>
       <c r="D352" t="n">
-        <v>0</v>
+        <v>-3.469446951953614e-18</v>
       </c>
       <c r="E352" t="inlineStr"/>
       <c r="F352" t="inlineStr">
@@ -12036,10 +12036,10 @@
         <v>0.003249918752031199</v>
       </c>
       <c r="C353" t="n">
-        <v>0.0032499187520312</v>
+        <v>0.003249918752031199</v>
       </c>
       <c r="D353" t="n">
-        <v>-4.336808689942018e-19</v>
+        <v>0</v>
       </c>
       <c r="E353" t="inlineStr"/>
       <c r="F353" t="inlineStr">
@@ -12100,10 +12100,10 @@
         <v>0.003420887071406102</v>
       </c>
       <c r="C355" t="n">
-        <v>0.003420887071406102</v>
+        <v>0.003420887071406103</v>
       </c>
       <c r="D355" t="n">
-        <v>0</v>
+        <v>-4.336808689942018e-19</v>
       </c>
       <c r="E355" t="inlineStr"/>
       <c r="F355" t="inlineStr">
@@ -12167,7 +12167,7 @@
         <v>0.0003774771940861906</v>
       </c>
       <c r="D357" t="n">
-        <v>5.421010862427522e-20</v>
+        <v>0</v>
       </c>
       <c r="E357" t="inlineStr"/>
       <c r="F357" t="inlineStr">
@@ -12260,10 +12260,10 @@
         <v>0.00528153644696639</v>
       </c>
       <c r="C360" t="n">
-        <v>0.005281536446966391</v>
+        <v>0.00528153644696639</v>
       </c>
       <c r="D360" t="n">
-        <v>-8.673617379884035e-19</v>
+        <v>0</v>
       </c>
       <c r="E360" t="inlineStr"/>
       <c r="F360" t="inlineStr">
@@ -12292,10 +12292,10 @@
         <v>0.007606490872210953</v>
       </c>
       <c r="C361" t="n">
-        <v>0.007606490872210954</v>
+        <v>0.007606490872210955</v>
       </c>
       <c r="D361" t="n">
-        <v>-8.673617379884035e-19</v>
+        <v>-1.734723475976807e-18</v>
       </c>
       <c r="E361" t="inlineStr"/>
       <c r="F361" t="inlineStr">
@@ -12740,10 +12740,10 @@
         <v>0.008477508650519031</v>
       </c>
       <c r="C375" t="n">
-        <v>0.008477508650519033</v>
+        <v>0.008477508650519031</v>
       </c>
       <c r="D375" t="n">
-        <v>-1.734723475976807e-18</v>
+        <v>0</v>
       </c>
       <c r="E375" t="inlineStr"/>
       <c r="F375" t="inlineStr">
@@ -12804,10 +12804,10 @@
         <v>0.009529411764705882</v>
       </c>
       <c r="C377" t="n">
-        <v>0.009529411764705882</v>
+        <v>0.009529411764705883</v>
       </c>
       <c r="D377" t="n">
-        <v>0</v>
+        <v>-1.734723475976807e-18</v>
       </c>
       <c r="E377" t="inlineStr"/>
       <c r="F377" t="inlineStr">
@@ -12984,10 +12984,10 @@
         <v>0.005227781926811053</v>
       </c>
       <c r="C383" t="n">
-        <v>0.005227781926811053</v>
+        <v>0.005227781926811052</v>
       </c>
       <c r="D383" t="n">
-        <v>0</v>
+        <v>8.673617379884035e-19</v>
       </c>
       <c r="E383" t="inlineStr"/>
       <c r="F383" t="inlineStr"/>
@@ -13236,10 +13236,10 @@
         <v>0.02894642215030565</v>
       </c>
       <c r="C392" t="n">
-        <v>0.02894642215030565</v>
+        <v>0.02894642215030564</v>
       </c>
       <c r="D392" t="n">
-        <v>0</v>
+        <v>3.469446951953614e-18</v>
       </c>
       <c r="E392" t="inlineStr"/>
       <c r="F392" t="inlineStr"/>
@@ -14636,10 +14636,10 @@
         <v>0.0004001600640256103</v>
       </c>
       <c r="C442" t="n">
-        <v>0.0004001600640256103</v>
+        <v>0.0004001600640256102</v>
       </c>
       <c r="D442" t="n">
-        <v>0</v>
+        <v>5.421010862427522e-20</v>
       </c>
       <c r="E442" t="inlineStr"/>
       <c r="F442" t="inlineStr"/>
@@ -15031,7 +15031,7 @@
         <v>0.02267290126141801</v>
       </c>
       <c r="D456" t="n">
-        <v>-3.469446951953614e-18</v>
+        <v>0</v>
       </c>
       <c r="E456" t="inlineStr"/>
       <c r="F456" t="inlineStr"/>
@@ -15199,7 +15199,7 @@
         <v>0.001479289940828402</v>
       </c>
       <c r="D462" t="n">
-        <v>0</v>
+        <v>2.168404344971009e-19</v>
       </c>
       <c r="E462" t="inlineStr"/>
       <c r="F462" t="inlineStr"/>
@@ -16876,10 +16876,10 @@
         <v>0.00931430836305985</v>
       </c>
       <c r="C522" t="n">
-        <v>0.00931430836305985</v>
+        <v>0.009314308363059848</v>
       </c>
       <c r="D522" t="n">
-        <v>0</v>
+        <v>1.734723475976807e-18</v>
       </c>
       <c r="E522" t="inlineStr"/>
       <c r="F522" t="inlineStr"/>
@@ -17411,7 +17411,7 @@
         <v>0.01087958694449567</v>
       </c>
       <c r="D541" t="n">
-        <v>0</v>
+        <v>-3.469446951953614e-18</v>
       </c>
       <c r="E541" t="inlineStr"/>
       <c r="F541" t="inlineStr"/>
@@ -17604,10 +17604,10 @@
         <v>0.003249918752031199</v>
       </c>
       <c r="C548" t="n">
-        <v>0.0032499187520312</v>
+        <v>0.003249918752031199</v>
       </c>
       <c r="D548" t="n">
-        <v>-4.336808689942018e-19</v>
+        <v>0</v>
       </c>
       <c r="E548" t="inlineStr"/>
       <c r="F548" t="inlineStr"/>
@@ -17660,10 +17660,10 @@
         <v>0.003420887071406102</v>
       </c>
       <c r="C550" t="n">
-        <v>0.003420887071406102</v>
+        <v>0.003420887071406103</v>
       </c>
       <c r="D550" t="n">
-        <v>0</v>
+        <v>-4.336808689942018e-19</v>
       </c>
       <c r="E550" t="inlineStr"/>
       <c r="F550" t="inlineStr"/>
@@ -17887,7 +17887,7 @@
         <v>0.0003774771940861906</v>
       </c>
       <c r="D558" t="n">
-        <v>5.421010862427522e-20</v>
+        <v>0</v>
       </c>
       <c r="E558" t="inlineStr"/>
       <c r="F558" t="inlineStr"/>
@@ -18080,10 +18080,10 @@
         <v>0.002251935256861365</v>
       </c>
       <c r="C565" t="n">
-        <v>0.002251935256861365</v>
+        <v>0.002251935256861366</v>
       </c>
       <c r="D565" t="n">
-        <v>0</v>
+        <v>-4.336808689942018e-19</v>
       </c>
       <c r="E565" t="inlineStr"/>
       <c r="F565" t="inlineStr"/>
@@ -18136,10 +18136,10 @@
         <v>0.00528153644696639</v>
       </c>
       <c r="C567" t="n">
-        <v>0.005281536446966391</v>
+        <v>0.00528153644696639</v>
       </c>
       <c r="D567" t="n">
-        <v>-8.673617379884035e-19</v>
+        <v>0</v>
       </c>
       <c r="E567" t="inlineStr"/>
       <c r="F567" t="inlineStr"/>
@@ -18164,10 +18164,10 @@
         <v>0.007606490872210953</v>
       </c>
       <c r="C568" t="n">
-        <v>0.007606490872210954</v>
+        <v>0.007606490872210955</v>
       </c>
       <c r="D568" t="n">
-        <v>-8.673617379884035e-19</v>
+        <v>-1.734723475976807e-18</v>
       </c>
       <c r="E568" t="inlineStr"/>
       <c r="F568" t="inlineStr"/>
@@ -18643,7 +18643,7 @@
         <v>0.003572615486872715</v>
       </c>
       <c r="D585" t="n">
-        <v>0</v>
+        <v>4.336808689942018e-19</v>
       </c>
       <c r="E585" t="inlineStr"/>
       <c r="F585" t="inlineStr"/>
@@ -21664,10 +21664,10 @@
         <v>0.008477508650519031</v>
       </c>
       <c r="C693" t="n">
-        <v>0.008477508650519033</v>
+        <v>0.008477508650519031</v>
       </c>
       <c r="D693" t="n">
-        <v>-1.734723475976807e-18</v>
+        <v>0</v>
       </c>
       <c r="E693" t="inlineStr"/>
       <c r="F693" t="inlineStr"/>
@@ -21972,10 +21972,10 @@
         <v>0.006896551724137931</v>
       </c>
       <c r="C704" t="n">
-        <v>0.00689655172413793</v>
+        <v>0.006896551724137929</v>
       </c>
       <c r="D704" t="n">
-        <v>8.673617379884035e-19</v>
+        <v>1.734723475976807e-18</v>
       </c>
       <c r="E704" t="inlineStr"/>
       <c r="F704" t="inlineStr"/>
@@ -22031,7 +22031,7 @@
         <v>0.01865847897968824</v>
       </c>
       <c r="D706" t="n">
-        <v>3.469446951953614e-18</v>
+        <v>0</v>
       </c>
       <c r="E706" t="inlineStr"/>
       <c r="F706" t="inlineStr"/>
@@ -22143,7 +22143,7 @@
         <v>0.002130681818181818</v>
       </c>
       <c r="D710" t="n">
-        <v>0</v>
+        <v>-4.336808689942018e-19</v>
       </c>
       <c r="E710" t="inlineStr"/>
       <c r="F710" t="inlineStr"/>
@@ -22644,10 +22644,10 @@
         <v>0.009529411764705882</v>
       </c>
       <c r="C728" t="n">
-        <v>0.009529411764705882</v>
+        <v>0.009529411764705883</v>
       </c>
       <c r="D728" t="n">
-        <v>0</v>
+        <v>-1.734723475976807e-18</v>
       </c>
       <c r="E728" t="inlineStr"/>
       <c r="F728" t="inlineStr"/>

</xml_diff>

<commit_message>
rerunning singleset stuff, got the v-gene decomp equation wrong the first time rip
</commit_message>
<xml_diff>
--- a/Final_Figures_and_Sheets_Singleset/Kb_jgene_decomposition_CDR3a.xlsx
+++ b/Final_Figures_and_Sheets_Singleset/Kb_jgene_decomposition_CDR3a.xlsx
@@ -480,10 +480,10 @@
         <v>0.1538168665524462</v>
       </c>
       <c r="C2" t="n">
-        <v>0.157910521941062</v>
+        <v>0.1538168665524462</v>
       </c>
       <c r="D2" t="n">
-        <v>-0.00409365538861578</v>
+        <v>0</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -516,10 +516,10 @@
         <v>0.2358513779527559</v>
       </c>
       <c r="C3" t="n">
-        <v>0.2408596462673611</v>
+        <v>0.2358513779527559</v>
       </c>
       <c r="D3" t="n">
-        <v>-0.005008268314605213</v>
+        <v>0</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -552,10 +552,10 @@
         <v>0.1377995642701525</v>
       </c>
       <c r="C4" t="n">
-        <v>0.142569321051155</v>
+        <v>0.1377995642701525</v>
       </c>
       <c r="D4" t="n">
-        <v>-0.004769756781002499</v>
+        <v>0</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -588,10 +588,10 @@
         <v>0.07772743116068316</v>
       </c>
       <c r="C5" t="n">
-        <v>0.08191856235485041</v>
+        <v>0.07772743116068315</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.004191131194167252</v>
+        <v>1.387778780781446e-17</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -624,10 +624,10 @@
         <v>0.1247199402539208</v>
       </c>
       <c r="C6" t="n">
-        <v>0.130001849112426</v>
+        <v>0.1247199402539208</v>
       </c>
       <c r="D6" t="n">
-        <v>-0.005281908858505213</v>
+        <v>-1.387778780781446e-17</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -660,10 +660,10 @@
         <v>0.1424242424242424</v>
       </c>
       <c r="C7" t="n">
-        <v>0.1471861471861472</v>
+        <v>0.1424242424242424</v>
       </c>
       <c r="D7" t="n">
-        <v>-0.004761904761904745</v>
+        <v>0</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -696,10 +696,10 @@
         <v>0.06577636037472594</v>
       </c>
       <c r="C8" t="n">
-        <v>0.06880713891032504</v>
+        <v>0.06577636037472592</v>
       </c>
       <c r="D8" t="n">
-        <v>-0.003030778535599105</v>
+        <v>1.387778780781446e-17</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -732,10 +732,10 @@
         <v>0.1761255821976885</v>
       </c>
       <c r="C9" t="n">
-        <v>0.1778074216383862</v>
+        <v>0.1761255821976885</v>
       </c>
       <c r="D9" t="n">
-        <v>-0.001681839440697747</v>
+        <v>-2.775557561562891e-17</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -768,10 +768,10 @@
         <v>0.02998084291187739</v>
       </c>
       <c r="C10" t="n">
-        <v>0.03216463335845025</v>
+        <v>0.0299808429118774</v>
       </c>
       <c r="D10" t="n">
-        <v>-0.002183790446572853</v>
+        <v>-6.938893903907228e-18</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -804,10 +804,10 @@
         <v>0.09842064714946071</v>
       </c>
       <c r="C11" t="n">
-        <v>0.1003502297768076</v>
+        <v>0.09842064714946068</v>
       </c>
       <c r="D11" t="n">
-        <v>-0.001929582627346924</v>
+        <v>2.775557561562891e-17</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -840,10 +840,10 @@
         <v>0.265563749916949</v>
       </c>
       <c r="C12" t="n">
-        <v>0.267768968623989</v>
+        <v>0.2655637499169491</v>
       </c>
       <c r="D12" t="n">
-        <v>-0.002205218707039991</v>
+        <v>-5.551115123125783e-17</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -876,10 +876,10 @@
         <v>0.1304592843054382</v>
       </c>
       <c r="C13" t="n">
-        <v>0.1329453958252264</v>
+        <v>0.1304592843054382</v>
       </c>
       <c r="D13" t="n">
-        <v>-0.002486111519788281</v>
+        <v>0</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -912,10 +912,10 @@
         <v>0.2271264646955255</v>
       </c>
       <c r="C14" t="n">
-        <v>0.2296512553380685</v>
+        <v>0.2271264646955255</v>
       </c>
       <c r="D14" t="n">
-        <v>-0.002524790642543073</v>
+        <v>0</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -948,10 +948,10 @@
         <v>0.1459243923012039</v>
       </c>
       <c r="C15" t="n">
-        <v>0.1482172894012702</v>
+        <v>0.1459243923012039</v>
       </c>
       <c r="D15" t="n">
-        <v>-0.002292897100066332</v>
+        <v>5.551115123125783e-17</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -984,10 +984,10 @@
         <v>0.03009971111732364</v>
       </c>
       <c r="C16" t="n">
-        <v>0.03201314065782301</v>
+        <v>0.03009971111732366</v>
       </c>
       <c r="D16" t="n">
-        <v>-0.001913429540499372</v>
+        <v>-1.387778780781446e-17</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -1020,10 +1020,10 @@
         <v>0.1496009821976673</v>
       </c>
       <c r="C17" t="n">
-        <v>0.152915964628194</v>
+        <v>0.1496009821976673</v>
       </c>
       <c r="D17" t="n">
-        <v>-0.003314982430526747</v>
+        <v>2.775557561562891e-17</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -1056,10 +1056,10 @@
         <v>0.06780617592517939</v>
       </c>
       <c r="C18" t="n">
-        <v>0.07110171980985953</v>
+        <v>0.06780617592517939</v>
       </c>
       <c r="D18" t="n">
-        <v>-0.003295543884680147</v>
+        <v>0</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -1092,10 +1092,10 @@
         <v>0.06132897603485839</v>
       </c>
       <c r="C19" t="n">
-        <v>0.06450938622301175</v>
+        <v>0.06132897603485838</v>
       </c>
       <c r="D19" t="n">
-        <v>-0.003180410188153363</v>
+        <v>6.938893903907228e-18</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -1128,10 +1128,10 @@
         <v>0.2442278860569715</v>
       </c>
       <c r="C20" t="n">
-        <v>0.2487118509710662</v>
+        <v>0.2442278860569716</v>
       </c>
       <c r="D20" t="n">
-        <v>-0.004483964914094668</v>
+        <v>-5.551115123125783e-17</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -1164,10 +1164,10 @@
         <v>0.399400299850075</v>
       </c>
       <c r="C21" t="n">
-        <v>0.4024841726387505</v>
+        <v>0.399400299850075</v>
       </c>
       <c r="D21" t="n">
-        <v>-0.003083872788675557</v>
+        <v>0</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -1200,10 +1200,10 @@
         <v>0.06048387096774194</v>
       </c>
       <c r="C22" t="n">
-        <v>0.06822620738636365</v>
+        <v>0.06048387096774193</v>
       </c>
       <c r="D22" t="n">
-        <v>-0.007742336418621709</v>
+        <v>6.938893903907228e-18</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -1236,10 +1236,10 @@
         <v>0.322623495226235</v>
       </c>
       <c r="C23" t="n">
-        <v>0.3244133215269579</v>
+        <v>0.322623495226235</v>
       </c>
       <c r="D23" t="n">
-        <v>-0.001789826300722941</v>
+        <v>0</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -1272,10 +1272,10 @@
         <v>0.2559339525283797</v>
       </c>
       <c r="C24" t="n">
-        <v>0.2584015954526719</v>
+        <v>0.2559339525283797</v>
       </c>
       <c r="D24" t="n">
-        <v>-0.002467642924292135</v>
+        <v>5.551115123125783e-17</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -1308,10 +1308,10 @@
         <v>0.06773211567732115</v>
       </c>
       <c r="C25" t="n">
-        <v>0.07294136713352325</v>
+        <v>0.06773211567732115</v>
       </c>
       <c r="D25" t="n">
-        <v>-0.005209251456202102</v>
+        <v>0</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -1344,10 +1344,10 @@
         <v>0.1044444444444445</v>
       </c>
       <c r="C26" t="n">
-        <v>0.1086015513897867</v>
+        <v>0.1044444444444444</v>
       </c>
       <c r="D26" t="n">
-        <v>-0.004157106945342229</v>
+        <v>1.387778780781446e-17</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -1380,10 +1380,10 @@
         <v>0.0969187675070028</v>
       </c>
       <c r="C27" t="n">
-        <v>0.1038754325259516</v>
+        <v>0.0969187675070028</v>
       </c>
       <c r="D27" t="n">
-        <v>-0.00695666501894876</v>
+        <v>0</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1416,10 +1416,10 @@
         <v>0.2727511146079203</v>
       </c>
       <c r="C28" t="n">
-        <v>0.2769650483437391</v>
+        <v>0.2727511146079202</v>
       </c>
       <c r="D28" t="n">
-        <v>-0.004213933735818798</v>
+        <v>1.110223024625157e-16</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1671,7 +1671,7 @@
         <v>0.001850328947368421</v>
       </c>
       <c r="D35" t="n">
-        <v>-2.168404344971009e-19</v>
+        <v>0</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1923,7 +1923,7 @@
         <v>0.02267290126141801</v>
       </c>
       <c r="D42" t="n">
-        <v>0</v>
+        <v>-3.469446951953614e-18</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -2028,10 +2028,10 @@
         <v>0.00931430836305985</v>
       </c>
       <c r="C45" t="n">
-        <v>0.009314308363059848</v>
+        <v>0.00931430836305985</v>
       </c>
       <c r="D45" t="n">
-        <v>1.734723475976807e-18</v>
+        <v>0</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -2067,7 +2067,7 @@
         <v>0.01087958694449567</v>
       </c>
       <c r="D46" t="n">
-        <v>-3.469446951953614e-18</v>
+        <v>0</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -2283,7 +2283,7 @@
         <v>0.1304155614500442</v>
       </c>
       <c r="D52" t="n">
-        <v>0</v>
+        <v>-2.775557561562891e-17</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -2355,7 +2355,7 @@
         <v>0.1730523627075351</v>
       </c>
       <c r="D54" t="n">
-        <v>0</v>
+        <v>2.775557561562891e-17</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -2424,10 +2424,10 @@
         <v>0.1031601534560114</v>
       </c>
       <c r="C56" t="n">
-        <v>0.1031601534560114</v>
+        <v>0.1031601534560115</v>
       </c>
       <c r="D56" t="n">
-        <v>0</v>
+        <v>-1.387778780781446e-17</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -2676,10 +2676,10 @@
         <v>0.008084172895677607</v>
       </c>
       <c r="C63" t="n">
-        <v>0.008084172895677607</v>
+        <v>0.008084172895677609</v>
       </c>
       <c r="D63" t="n">
-        <v>0</v>
+        <v>-1.734723475976807e-18</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -3075,7 +3075,7 @@
         <v>0.002130681818181818</v>
       </c>
       <c r="D74" t="n">
-        <v>-4.336808689942018e-19</v>
+        <v>0</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -3687,7 +3687,7 @@
         <v>0.001850328947368421</v>
       </c>
       <c r="D92" t="n">
-        <v>-2.168404344971009e-19</v>
+        <v>0</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -4103,7 +4103,7 @@
         <v>0.02267290126141801</v>
       </c>
       <c r="D105" t="n">
-        <v>0</v>
+        <v>-3.469446951953614e-18</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -4484,10 +4484,10 @@
         <v>0.00931430836305985</v>
       </c>
       <c r="C117" t="n">
-        <v>0.009314308363059848</v>
+        <v>0.00931430836305985</v>
       </c>
       <c r="D117" t="n">
-        <v>1.734723475976807e-18</v>
+        <v>0</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -4519,7 +4519,7 @@
         <v>0.01087958694449567</v>
       </c>
       <c r="D118" t="n">
-        <v>-3.469446951953614e-18</v>
+        <v>0</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -4775,7 +4775,7 @@
         <v>0.003572615486872715</v>
       </c>
       <c r="D126" t="n">
-        <v>4.336808689942018e-19</v>
+        <v>0</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -4807,7 +4807,7 @@
         <v>0.1304155614500442</v>
       </c>
       <c r="D127" t="n">
-        <v>0</v>
+        <v>-2.775557561562891e-17</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -4871,7 +4871,7 @@
         <v>0.1730523627075351</v>
       </c>
       <c r="D129" t="n">
-        <v>0</v>
+        <v>2.775557561562891e-17</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -5028,10 +5028,10 @@
         <v>0.1031601534560114</v>
       </c>
       <c r="C134" t="n">
-        <v>0.1031601534560114</v>
+        <v>0.1031601534560115</v>
       </c>
       <c r="D134" t="n">
-        <v>0</v>
+        <v>-1.387778780781446e-17</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -5636,10 +5636,10 @@
         <v>0.008084172895677607</v>
       </c>
       <c r="C153" t="n">
-        <v>0.008084172895677607</v>
+        <v>0.008084172895677609</v>
       </c>
       <c r="D153" t="n">
-        <v>0</v>
+        <v>-1.734723475976807e-18</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -6183,7 +6183,7 @@
         <v>0.002130681818181818</v>
       </c>
       <c r="D170" t="n">
-        <v>-4.336808689942018e-19</v>
+        <v>0</v>
       </c>
       <c r="E170" t="inlineStr">
         <is>
@@ -7431,7 +7431,7 @@
         <v>0.001850328947368421</v>
       </c>
       <c r="D209" t="n">
-        <v>-2.168404344971009e-19</v>
+        <v>0</v>
       </c>
       <c r="E209" t="inlineStr"/>
       <c r="F209" t="inlineStr">
@@ -8423,7 +8423,7 @@
         <v>0.02267290126141801</v>
       </c>
       <c r="D240" t="n">
-        <v>0</v>
+        <v>-3.469446951953614e-18</v>
       </c>
       <c r="E240" t="inlineStr"/>
       <c r="F240" t="inlineStr">
@@ -8519,7 +8519,7 @@
         <v>0.001479289940828402</v>
       </c>
       <c r="D243" t="n">
-        <v>2.168404344971009e-19</v>
+        <v>0</v>
       </c>
       <c r="E243" t="inlineStr"/>
       <c r="F243" t="inlineStr">
@@ -9991,7 +9991,7 @@
         <v>0.1304155614500442</v>
       </c>
       <c r="D289" t="n">
-        <v>0</v>
+        <v>-2.775557561562891e-17</v>
       </c>
       <c r="E289" t="inlineStr"/>
       <c r="F289" t="inlineStr">
@@ -10055,7 +10055,7 @@
         <v>0.1730523627075351</v>
       </c>
       <c r="D291" t="n">
-        <v>0</v>
+        <v>2.775557561562891e-17</v>
       </c>
       <c r="E291" t="inlineStr"/>
       <c r="F291" t="inlineStr">
@@ -10308,10 +10308,10 @@
         <v>0.1031601534560114</v>
       </c>
       <c r="C299" t="n">
-        <v>0.1031601534560114</v>
+        <v>0.1031601534560115</v>
       </c>
       <c r="D299" t="n">
-        <v>0</v>
+        <v>-1.387778780781446e-17</v>
       </c>
       <c r="E299" t="inlineStr"/>
       <c r="F299" t="inlineStr">
@@ -11559,7 +11559,7 @@
         <v>0.002130681818181818</v>
       </c>
       <c r="D338" t="n">
-        <v>-4.336808689942018e-19</v>
+        <v>0</v>
       </c>
       <c r="E338" t="inlineStr"/>
       <c r="F338" t="inlineStr">
@@ -11780,10 +11780,10 @@
         <v>0.00931430836305985</v>
       </c>
       <c r="C345" t="n">
-        <v>0.009314308363059848</v>
+        <v>0.00931430836305985</v>
       </c>
       <c r="D345" t="n">
-        <v>1.734723475976807e-18</v>
+        <v>0</v>
       </c>
       <c r="E345" t="inlineStr"/>
       <c r="F345" t="inlineStr">
@@ -12007,7 +12007,7 @@
         <v>0.01087958694449567</v>
       </c>
       <c r="D352" t="n">
-        <v>-3.469446951953614e-18</v>
+        <v>0</v>
       </c>
       <c r="E352" t="inlineStr"/>
       <c r="F352" t="inlineStr">
@@ -12039,7 +12039,7 @@
         <v>0.003249918752031199</v>
       </c>
       <c r="D353" t="n">
-        <v>0</v>
+        <v>4.336808689942018e-19</v>
       </c>
       <c r="E353" t="inlineStr"/>
       <c r="F353" t="inlineStr">
@@ -12167,7 +12167,7 @@
         <v>0.0003774771940861906</v>
       </c>
       <c r="D357" t="n">
-        <v>0</v>
+        <v>5.421010862427522e-20</v>
       </c>
       <c r="E357" t="inlineStr"/>
       <c r="F357" t="inlineStr">
@@ -12292,10 +12292,10 @@
         <v>0.007606490872210953</v>
       </c>
       <c r="C361" t="n">
-        <v>0.007606490872210955</v>
+        <v>0.007606490872210954</v>
       </c>
       <c r="D361" t="n">
-        <v>-1.734723475976807e-18</v>
+        <v>-8.673617379884035e-19</v>
       </c>
       <c r="E361" t="inlineStr"/>
       <c r="F361" t="inlineStr">
@@ -12452,10 +12452,10 @@
         <v>0.008084172895677607</v>
       </c>
       <c r="C366" t="n">
-        <v>0.008084172895677607</v>
+        <v>0.008084172895677609</v>
       </c>
       <c r="D366" t="n">
-        <v>0</v>
+        <v>-1.734723475976807e-18</v>
       </c>
       <c r="E366" t="inlineStr"/>
       <c r="F366" t="inlineStr">
@@ -12740,10 +12740,10 @@
         <v>0.008477508650519031</v>
       </c>
       <c r="C375" t="n">
-        <v>0.008477508650519031</v>
+        <v>0.008477508650519033</v>
       </c>
       <c r="D375" t="n">
-        <v>0</v>
+        <v>-1.734723475976807e-18</v>
       </c>
       <c r="E375" t="inlineStr"/>
       <c r="F375" t="inlineStr">
@@ -13659,7 +13659,7 @@
         <v>0.001850328947368421</v>
       </c>
       <c r="D407" t="n">
-        <v>-2.168404344971009e-19</v>
+        <v>0</v>
       </c>
       <c r="E407" t="inlineStr"/>
       <c r="F407" t="inlineStr"/>
@@ -15031,7 +15031,7 @@
         <v>0.02267290126141801</v>
       </c>
       <c r="D456" t="n">
-        <v>0</v>
+        <v>-3.469446951953614e-18</v>
       </c>
       <c r="E456" t="inlineStr"/>
       <c r="F456" t="inlineStr"/>
@@ -15199,7 +15199,7 @@
         <v>0.001479289940828402</v>
       </c>
       <c r="D462" t="n">
-        <v>2.168404344971009e-19</v>
+        <v>0</v>
       </c>
       <c r="E462" t="inlineStr"/>
       <c r="F462" t="inlineStr"/>
@@ -16876,10 +16876,10 @@
         <v>0.00931430836305985</v>
       </c>
       <c r="C522" t="n">
-        <v>0.009314308363059848</v>
+        <v>0.00931430836305985</v>
       </c>
       <c r="D522" t="n">
-        <v>1.734723475976807e-18</v>
+        <v>0</v>
       </c>
       <c r="E522" t="inlineStr"/>
       <c r="F522" t="inlineStr"/>
@@ -17411,7 +17411,7 @@
         <v>0.01087958694449567</v>
       </c>
       <c r="D541" t="n">
-        <v>-3.469446951953614e-18</v>
+        <v>0</v>
       </c>
       <c r="E541" t="inlineStr"/>
       <c r="F541" t="inlineStr"/>
@@ -17607,7 +17607,7 @@
         <v>0.003249918752031199</v>
       </c>
       <c r="D548" t="n">
-        <v>0</v>
+        <v>4.336808689942018e-19</v>
       </c>
       <c r="E548" t="inlineStr"/>
       <c r="F548" t="inlineStr"/>
@@ -17887,7 +17887,7 @@
         <v>0.0003774771940861906</v>
       </c>
       <c r="D558" t="n">
-        <v>0</v>
+        <v>5.421010862427522e-20</v>
       </c>
       <c r="E558" t="inlineStr"/>
       <c r="F558" t="inlineStr"/>
@@ -18164,10 +18164,10 @@
         <v>0.007606490872210953</v>
       </c>
       <c r="C568" t="n">
-        <v>0.007606490872210955</v>
+        <v>0.007606490872210954</v>
       </c>
       <c r="D568" t="n">
-        <v>-1.734723475976807e-18</v>
+        <v>-8.673617379884035e-19</v>
       </c>
       <c r="E568" t="inlineStr"/>
       <c r="F568" t="inlineStr"/>
@@ -18643,7 +18643,7 @@
         <v>0.003572615486872715</v>
       </c>
       <c r="D585" t="n">
-        <v>4.336808689942018e-19</v>
+        <v>0</v>
       </c>
       <c r="E585" t="inlineStr"/>
       <c r="F585" t="inlineStr"/>
@@ -18923,7 +18923,7 @@
         <v>0.1304155614500442</v>
       </c>
       <c r="D595" t="n">
-        <v>0</v>
+        <v>-2.775557561562891e-17</v>
       </c>
       <c r="E595" t="inlineStr"/>
       <c r="F595" t="inlineStr"/>
@@ -18979,7 +18979,7 @@
         <v>0.1730523627075351</v>
       </c>
       <c r="D597" t="n">
-        <v>0</v>
+        <v>2.775557561562891e-17</v>
       </c>
       <c r="E597" t="inlineStr"/>
       <c r="F597" t="inlineStr"/>
@@ -19368,10 +19368,10 @@
         <v>0.1031601534560114</v>
       </c>
       <c r="C611" t="n">
-        <v>0.1031601534560114</v>
+        <v>0.1031601534560115</v>
       </c>
       <c r="D611" t="n">
-        <v>0</v>
+        <v>-1.387778780781446e-17</v>
       </c>
       <c r="E611" t="inlineStr"/>
       <c r="F611" t="inlineStr"/>
@@ -20908,10 +20908,10 @@
         <v>0.008084172895677607</v>
       </c>
       <c r="C666" t="n">
-        <v>0.008084172895677607</v>
+        <v>0.008084172895677609</v>
       </c>
       <c r="D666" t="n">
-        <v>0</v>
+        <v>-1.734723475976807e-18</v>
       </c>
       <c r="E666" t="inlineStr"/>
       <c r="F666" t="inlineStr"/>
@@ -21664,10 +21664,10 @@
         <v>0.008477508650519031</v>
       </c>
       <c r="C693" t="n">
-        <v>0.008477508650519031</v>
+        <v>0.008477508650519033</v>
       </c>
       <c r="D693" t="n">
-        <v>0</v>
+        <v>-1.734723475976807e-18</v>
       </c>
       <c r="E693" t="inlineStr"/>
       <c r="F693" t="inlineStr"/>
@@ -22143,7 +22143,7 @@
         <v>0.002130681818181818</v>
       </c>
       <c r="D710" t="n">
-        <v>-4.336808689942018e-19</v>
+        <v>0</v>
       </c>
       <c r="E710" t="inlineStr"/>
       <c r="F710" t="inlineStr"/>
@@ -22728,10 +22728,10 @@
         <v>0.0001720323163889472</v>
       </c>
       <c r="C731" t="n">
-        <v>0.0001720348006511756</v>
+        <v>0.0001720051154309581</v>
       </c>
       <c r="D731" t="n">
-        <v>-2.484262228412025e-09</v>
+        <v>2.720095798909171e-08</v>
       </c>
       <c r="E731" t="inlineStr"/>
       <c r="F731" t="inlineStr"/>
@@ -22756,10 +22756,10 @@
         <v>6.190664724656162e-05</v>
       </c>
       <c r="C732" t="n">
-        <v>6.190231547701336e-05</v>
+        <v>6.189066493642178e-05</v>
       </c>
       <c r="D732" t="n">
-        <v>4.331769548257796e-09</v>
+        <v>1.598231013983829e-08</v>
       </c>
       <c r="E732" t="inlineStr"/>
       <c r="F732" t="inlineStr"/>

</xml_diff>

<commit_message>
ran it again with proper naming x
</commit_message>
<xml_diff>
--- a/Final_Figures_and_Sheets_Singleset/Kb_jgene_decomposition_CDR3a.xlsx
+++ b/Final_Figures_and_Sheets_Singleset/Kb_jgene_decomposition_CDR3a.xlsx
@@ -1671,7 +1671,7 @@
         <v>0.001850328947368421</v>
       </c>
       <c r="D35" t="n">
-        <v>0</v>
+        <v>-2.168404344971009e-19</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -2283,7 +2283,7 @@
         <v>0.1304155614500442</v>
       </c>
       <c r="D52" t="n">
-        <v>-2.775557561562891e-17</v>
+        <v>0</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -2355,7 +2355,7 @@
         <v>0.1730523627075351</v>
       </c>
       <c r="D54" t="n">
-        <v>2.775557561562891e-17</v>
+        <v>0</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -2424,10 +2424,10 @@
         <v>0.1031601534560114</v>
       </c>
       <c r="C56" t="n">
-        <v>0.1031601534560115</v>
+        <v>0.1031601534560114</v>
       </c>
       <c r="D56" t="n">
-        <v>-1.387778780781446e-17</v>
+        <v>0</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -2964,10 +2964,10 @@
         <v>0.006896551724137931</v>
       </c>
       <c r="C71" t="n">
-        <v>0.006896551724137929</v>
+        <v>0.00689655172413793</v>
       </c>
       <c r="D71" t="n">
-        <v>1.734723475976807e-18</v>
+        <v>8.673617379884035e-19</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -3288,10 +3288,10 @@
         <v>0.009529411764705882</v>
       </c>
       <c r="C80" t="n">
-        <v>0.009529411764705883</v>
+        <v>0.009529411764705882</v>
       </c>
       <c r="D80" t="n">
-        <v>-1.734723475976807e-18</v>
+        <v>0</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -3687,7 +3687,7 @@
         <v>0.001850328947368421</v>
       </c>
       <c r="D92" t="n">
-        <v>0</v>
+        <v>-2.168404344971009e-19</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -4807,7 +4807,7 @@
         <v>0.1304155614500442</v>
       </c>
       <c r="D127" t="n">
-        <v>-2.775557561562891e-17</v>
+        <v>0</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -4871,7 +4871,7 @@
         <v>0.1730523627075351</v>
       </c>
       <c r="D129" t="n">
-        <v>2.775557561562891e-17</v>
+        <v>0</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -5028,10 +5028,10 @@
         <v>0.1031601534560114</v>
       </c>
       <c r="C134" t="n">
-        <v>0.1031601534560115</v>
+        <v>0.1031601534560114</v>
       </c>
       <c r="D134" t="n">
-        <v>-1.387778780781446e-17</v>
+        <v>0</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -5988,10 +5988,10 @@
         <v>0.006896551724137931</v>
       </c>
       <c r="C164" t="n">
-        <v>0.006896551724137929</v>
+        <v>0.00689655172413793</v>
       </c>
       <c r="D164" t="n">
-        <v>1.734723475976807e-18</v>
+        <v>8.673617379884035e-19</v>
       </c>
       <c r="E164" t="inlineStr">
         <is>
@@ -6756,10 +6756,10 @@
         <v>0.009529411764705882</v>
       </c>
       <c r="C188" t="n">
-        <v>0.009529411764705883</v>
+        <v>0.009529411764705882</v>
       </c>
       <c r="D188" t="n">
-        <v>-1.734723475976807e-18</v>
+        <v>0</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -7431,7 +7431,7 @@
         <v>0.001850328947368421</v>
       </c>
       <c r="D209" t="n">
-        <v>0</v>
+        <v>-2.168404344971009e-19</v>
       </c>
       <c r="E209" t="inlineStr"/>
       <c r="F209" t="inlineStr">
@@ -9991,7 +9991,7 @@
         <v>0.1304155614500442</v>
       </c>
       <c r="D289" t="n">
-        <v>-2.775557561562891e-17</v>
+        <v>0</v>
       </c>
       <c r="E289" t="inlineStr"/>
       <c r="F289" t="inlineStr">
@@ -10055,7 +10055,7 @@
         <v>0.1730523627075351</v>
       </c>
       <c r="D291" t="n">
-        <v>2.775557561562891e-17</v>
+        <v>0</v>
       </c>
       <c r="E291" t="inlineStr"/>
       <c r="F291" t="inlineStr">
@@ -10308,10 +10308,10 @@
         <v>0.1031601534560114</v>
       </c>
       <c r="C299" t="n">
-        <v>0.1031601534560115</v>
+        <v>0.1031601534560114</v>
       </c>
       <c r="D299" t="n">
-        <v>-1.387778780781446e-17</v>
+        <v>0</v>
       </c>
       <c r="E299" t="inlineStr"/>
       <c r="F299" t="inlineStr">
@@ -11460,10 +11460,10 @@
         <v>0.006896551724137931</v>
       </c>
       <c r="C335" t="n">
-        <v>0.006896551724137929</v>
+        <v>0.00689655172413793</v>
       </c>
       <c r="D335" t="n">
-        <v>1.734723475976807e-18</v>
+        <v>8.673617379884035e-19</v>
       </c>
       <c r="E335" t="inlineStr"/>
       <c r="F335" t="inlineStr">
@@ -12039,7 +12039,7 @@
         <v>0.003249918752031199</v>
       </c>
       <c r="D353" t="n">
-        <v>4.336808689942018e-19</v>
+        <v>0</v>
       </c>
       <c r="E353" t="inlineStr"/>
       <c r="F353" t="inlineStr">
@@ -12100,10 +12100,10 @@
         <v>0.003420887071406102</v>
       </c>
       <c r="C355" t="n">
-        <v>0.003420887071406103</v>
+        <v>0.003420887071406102</v>
       </c>
       <c r="D355" t="n">
-        <v>-4.336808689942018e-19</v>
+        <v>0</v>
       </c>
       <c r="E355" t="inlineStr"/>
       <c r="F355" t="inlineStr">
@@ -12260,10 +12260,10 @@
         <v>0.00528153644696639</v>
       </c>
       <c r="C360" t="n">
-        <v>0.00528153644696639</v>
+        <v>0.005281536446966391</v>
       </c>
       <c r="D360" t="n">
-        <v>0</v>
+        <v>-8.673617379884035e-19</v>
       </c>
       <c r="E360" t="inlineStr"/>
       <c r="F360" t="inlineStr">
@@ -12804,10 +12804,10 @@
         <v>0.009529411764705882</v>
       </c>
       <c r="C377" t="n">
-        <v>0.009529411764705883</v>
+        <v>0.009529411764705882</v>
       </c>
       <c r="D377" t="n">
-        <v>-1.734723475976807e-18</v>
+        <v>0</v>
       </c>
       <c r="E377" t="inlineStr"/>
       <c r="F377" t="inlineStr">
@@ -13659,7 +13659,7 @@
         <v>0.001850328947368421</v>
       </c>
       <c r="D407" t="n">
-        <v>0</v>
+        <v>-2.168404344971009e-19</v>
       </c>
       <c r="E407" t="inlineStr"/>
       <c r="F407" t="inlineStr"/>
@@ -17607,7 +17607,7 @@
         <v>0.003249918752031199</v>
       </c>
       <c r="D548" t="n">
-        <v>4.336808689942018e-19</v>
+        <v>0</v>
       </c>
       <c r="E548" t="inlineStr"/>
       <c r="F548" t="inlineStr"/>
@@ -17660,10 +17660,10 @@
         <v>0.003420887071406102</v>
       </c>
       <c r="C550" t="n">
-        <v>0.003420887071406103</v>
+        <v>0.003420887071406102</v>
       </c>
       <c r="D550" t="n">
-        <v>-4.336808689942018e-19</v>
+        <v>0</v>
       </c>
       <c r="E550" t="inlineStr"/>
       <c r="F550" t="inlineStr"/>
@@ -18136,10 +18136,10 @@
         <v>0.00528153644696639</v>
       </c>
       <c r="C567" t="n">
-        <v>0.00528153644696639</v>
+        <v>0.005281536446966391</v>
       </c>
       <c r="D567" t="n">
-        <v>0</v>
+        <v>-8.673617379884035e-19</v>
       </c>
       <c r="E567" t="inlineStr"/>
       <c r="F567" t="inlineStr"/>
@@ -18923,7 +18923,7 @@
         <v>0.1304155614500442</v>
       </c>
       <c r="D595" t="n">
-        <v>-2.775557561562891e-17</v>
+        <v>0</v>
       </c>
       <c r="E595" t="inlineStr"/>
       <c r="F595" t="inlineStr"/>
@@ -18979,7 +18979,7 @@
         <v>0.1730523627075351</v>
       </c>
       <c r="D597" t="n">
-        <v>2.775557561562891e-17</v>
+        <v>0</v>
       </c>
       <c r="E597" t="inlineStr"/>
       <c r="F597" t="inlineStr"/>
@@ -19368,10 +19368,10 @@
         <v>0.1031601534560114</v>
       </c>
       <c r="C611" t="n">
-        <v>0.1031601534560115</v>
+        <v>0.1031601534560114</v>
       </c>
       <c r="D611" t="n">
-        <v>-1.387778780781446e-17</v>
+        <v>0</v>
       </c>
       <c r="E611" t="inlineStr"/>
       <c r="F611" t="inlineStr"/>
@@ -21972,10 +21972,10 @@
         <v>0.006896551724137931</v>
       </c>
       <c r="C704" t="n">
-        <v>0.006896551724137929</v>
+        <v>0.00689655172413793</v>
       </c>
       <c r="D704" t="n">
-        <v>1.734723475976807e-18</v>
+        <v>8.673617379884035e-19</v>
       </c>
       <c r="E704" t="inlineStr"/>
       <c r="F704" t="inlineStr"/>
@@ -22644,10 +22644,10 @@
         <v>0.009529411764705882</v>
       </c>
       <c r="C728" t="n">
-        <v>0.009529411764705883</v>
+        <v>0.009529411764705882</v>
       </c>
       <c r="D728" t="n">
-        <v>-1.734723475976807e-18</v>
+        <v>0</v>
       </c>
       <c r="E728" t="inlineStr"/>
       <c r="F728" t="inlineStr"/>

</xml_diff>